<commit_message>
Normalize department casing in Trespass catalog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Eo9b23QXeMg42JisPjnCY
</commit_message>
<xml_diff>
--- a/Trespass_Catalog.xlsx
+++ b/Trespass_Catalog.xlsx
@@ -1357,7 +1357,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>swim</t>
+          <t>Swim</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>rucksacks</t>
+          <t>Rucksacks</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>cycling</t>
+          <t>Cycling</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>swim</t>
+          <t>Swim</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>snowsports</t>
+          <t>Snowsports</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>footwear</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>snowsports</t>
+          <t>Snowsports</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>rucksacks</t>
+          <t>Rucksacks</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>rucksacks</t>
+          <t>Rucksacks</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>rucksacks</t>
+          <t>Rucksacks</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>snowsports</t>
+          <t>Snowsports</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>rucksacks</t>
+          <t>Rucksacks</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>swim</t>
+          <t>Swim</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>swim</t>
+          <t>Swim</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4719,7 +4719,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6052,7 +6052,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -6527,7 +6527,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -6607,7 +6607,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -6874,7 +6874,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -7157,7 +7157,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -7237,7 +7237,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -7403,7 +7403,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -7669,7 +7669,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>rucksacks</t>
+          <t>Rucksacks</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -7818,7 +7818,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -8022,7 +8022,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -8161,7 +8161,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -8358,7 +8358,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -8512,7 +8512,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -8549,7 +8549,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -8660,7 +8660,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -8851,7 +8851,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -8968,7 +8968,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -9140,7 +9140,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -9177,7 +9177,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -9325,7 +9325,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -9362,7 +9362,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -9436,7 +9436,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -9479,7 +9479,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -9553,7 +9553,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -9707,7 +9707,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -9856,7 +9856,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9973,7 +9973,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -10170,7 +10170,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -10213,7 +10213,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -10299,7 +10299,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -10454,7 +10454,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -10528,7 +10528,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -10645,7 +10645,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -10682,7 +10682,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -10768,7 +10768,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -10805,7 +10805,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -11045,7 +11045,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -11131,7 +11131,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>camping</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -11168,7 +11168,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -11482,7 +11482,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11525,7 +11525,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11611,7 +11611,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11723,7 +11723,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11920,7 +11920,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11963,7 +11963,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -12000,7 +12000,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -12117,7 +12117,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -12154,7 +12154,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -12356,7 +12356,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -12442,7 +12442,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -12479,7 +12479,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -12522,7 +12522,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12602,7 +12602,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12682,7 +12682,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12971,7 +12971,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -13014,7 +13014,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -13088,7 +13088,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -13125,7 +13125,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -13199,7 +13199,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -13322,7 +13322,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -13470,7 +13470,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -13544,7 +13544,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -13613,7 +13613,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13650,7 +13650,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13687,7 +13687,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -13761,7 +13761,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -13798,7 +13798,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -13835,7 +13835,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -13872,7 +13872,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -13952,7 +13952,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>kids</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">

</xml_diff>